<commit_message>
Auto: Week 25/2026 data extracted from PDFs
</commit_message>
<xml_diff>
--- a/Gulf_Dashboard_W25_2026.xlsx
+++ b/Gulf_Dashboard_W25_2026.xlsx
@@ -750,232 +750,784 @@
       <c r="E11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>PRJ-013</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>GCE</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>➢ GCE-001-C-022-UEA-101 Boiler&amp;FGT ground beam plan TOB EL+0.15 not have detail drain line
+Concern (delay)
+Detailsregardingthedrainpiesize,routing,anddepth werenotfound..
+Follow up and urge EPC to resolve the issues in the daily meeting.
+If you return late, that point will be blocked (This is a recommendation from OE.)
+EPC are urging designer&amp;EPC engineering solve the problem of drawing.
+➢ GCE-001-E-106-00-006 cable route layout, and COM-001-E-106-UMA-101 Cable layout for STG building, the 2 versions do not match
+Thereareroutingconflicts in the STG building cable layout..
+Inform the EPC to solve the conflicts drawing soon.
+EPC &amp; STECON acknowledge.
+➢ GCE-001-C-022-UAE-201_Bunker pit ground floor framing plan EL +0.25 s the concern about the increased slope of 20 cm correct?
+The drawing needs to be fixed urgently within end of June
+Affect to plan slab ground floor
+Co-ordinated with civil team EPC and OE for follow up
+Summary of Safety Weekly Audit issues
+Total Issues 8 9 5
+since 03 Apr 2026 - Present 4-Jun 11-Jun 18-Jun 25-Jun
+(Every Tuesday morning)
+Series1 Series2
+Safety Audit issue Status Chart</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>SM EPC is urging its EPC design and engineering teams to provide the data.
+Safety &amp; Health:
+Management site walkdown
+Toolbox talk activity
+Safety induction training to new contractors​
+Weekly Inspect Safety​
+Weekly Random Alc. Test
+Environment &amp; CoP:
+Road cleaning (Campsite STECON/IEAT Road)
+Water spray to reduce dust
+Monitor noise during overtime work
+Activities CC/SC (*)
+Plan Actual Diff. Plan Actual Diff. Acc.Plan
+% % % % % % %
+Engineering 10.00% 67.58% 42.57% -25.01% 74.32% 44.16% 30.16% 80.30%
+Procurement 40.00% 71.12% 69.35% -1.77% 72.89% 70.86%
+Construction 40.00% 13.16% 8.16% -5.00% 14.29% 9.58 -4.71% 15.70%
+Commissioning 10.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00%
+Overall 100.00% 40.47% 35.26 -5.21% 42.30% 36.59% -5.71 44.06%
+** The data cut off every Friday of week</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>PRJ-014</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>GSE</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="2" t="inlineStr"/>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Bunker and surrounding: Foundation up to ground (including the surrounding room, underground grounding system).
+Boiler : Boiler steel structure.
+Flue gas treatment : Foundation work.
+STG &amp; ECB : Foundation up to ground (including the surrounding room, underground grounding system).
+Tipping hall: Pilling work and foundation.
+Concern (delay)
+Delay finish of bunker foundations up to ground level. Target on PMS 07 May 2026.
+Delay finish of STG foundations up to ground level. Target on PMS 25 May 2026.
+CEEC/STECON prepare catch-up plan for bunker and boiler foundation up to ground level
+CEEC/STECON will increase man power more than plan
+- This week (Finished : 2)
+- Total(Finished : 36)
+0 RFC , 3 NCR
+7 Stakeholder Engagement Plan Continue as plan
+8 SHE Plan for counting manpower working at site Manpower daily report have started to generating automatically at 7:00
+AM everyday by e-mail
+9 Status of EPC Foreigner staff and worker personal mandatory document Pending 27 prs. Plan to finish &lt;10 Jul 2026&gt;
+36 Safety Weekly Audit issue
+Total Issues
+(Since 2 Apr 2026 onwards)</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Activities CC/SC (*)
+Plan% Actual% Diff.% Plan% Actual% Diff.% Acc.Plan%
+Engineering 10% 67.58% 43.90% -23.68% 74.32% 45.48% -28.84% 80.30%
+Procurement 40% 71.12% 69.35% -1.77% 72.89% 70.86% -3.79% 74.39%
+Construction 40% 13.16% 10.70% -2.46% 14.29% 12.91% -1.38% 15.70%
+Commissioning 10% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00%
+Overall 100% 40.47% 36.41% -4.06% 42.30% 38.06% -4.25% 44.06%
+5 Maximum Quantity of Heavy Machinery at Site Inspection as period
+and keep related document
+6 Summary of SHE Weekly Audit issues Walk down
+- This week (Finished : 2)
+- Total(Finished : 36)
+0 RFC , 3 NCR
+7 Stakeholder Engagement Plan Continue as plan
+8 SHE Plan for counting manpower working at site Manpower daily report have started to generating automatically at 7:00
+AM everyday by e-mail
+9 Status of EPC Foreigner staff and worker personal mandatory document Pending 27 prs. Plan to finish &lt;10 Jul 2026&gt;
+Safety &amp; Health:
+• Safety Toolbox Talk before starting work and Mass Toolbox Talk and counting manpower
+• Safety training for newcomer</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>PRJ-015</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>KKE</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr"/>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>311-314 Refuse Bunker Super structure up to 35.5m elevation 9 May 26 23 Nov 26 Delay Start
+325-326 Tipping hall Foundation up to ground (Include piling work) 1 Feb 26 9 Jul 26 8 Feb 26 On going
+327 Tipping hall Super structure up to 13m elevation 10 Jul 26 19 Oct 26
+330-335 Boiler Island &amp; Auxiliary Equipment Foundation 5 Nov 25 14 Jul 26 8 Jan 26 On going
+346 Steam Turbine Generator &amp; Electrical Construction 18 Feb 26 3 Mar 27 8 Feb 26 On going
+408 Holding Pond and Emergency PondConstruction 23 May 26 20 Nov 26
+14 Boiler Arrival at site 12 Jun 26 12 Jun 26
+11 Incinerator Arrival at site 8 May 26 8 May 26 3 May 26 5 May 26 Completed
+15 Steam turbine Arrival at site 2 Oct 26 2 Oct 26
+62- Producing qualified water (Water Receiving date) 23 Feb 27 8 Mar 27
+EPC has adjusted the PMS to Rev.H to make the plan consistent with the actual work
+Completion of Concrete pouring for surrounding area Targeted by 16-17-JUL-2026
+Completion of Lift 2: Bunker Wall EL +1.0 to +5.45 Targeted by 28-29-Jun-2026
+Completed of Steel structure erection for Upper part Z1-Z6 at EL 11.3-41.6 m
+Commencement for FGT Equipment Bag filter erection.
+Partial handover (civil works) of Switchgear room in the STG &amp; EC Building, including all related areas required for the installation of 22 kV and 11 kV switchgear and
+power cables.
+Piling work for the Cooling Tower may affect Metek Company due to vibrations impacting its X-ray measuring equipment.
+127 Safety Weekly Audit issue status by weekly
+Total Issues</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Key Lookahead milestone:
+Bunker building: Concrete pouring for Lift 2 Wall EL +1.0 to +5.45 Targeted by 28-29-Jun-2026
+Concrete pouring for surrounding area Targeted by 16-17-JUL-2026
+Boiler &amp; Incinerator Erection: Steel structure erection for Upper part Z1-Z6 at EL 11.3-41.6 m
+FGT: Commencement for FGT Equipment Bag filter erection.
+STG &amp; ECB: Commencement of Slab for 22kV SWGR&amp;MCC Cable Trench at EL -0.70.
+The tower crane: Completed of installation Targeted by 3-4 Jul 2026
+Balance of Plant: Completed of pilling work Service water tank &amp; Fire water pump shelter
+Pre-conditions required: -
+Area of Concern: Piling work for the Cooling Tower may affect Metek Company due to vibrations
+impacting its X-ray measuring equipment.
+Issue to request HO support: -
+Completed of pilling work Service water tank &amp; Fire water pump shelter
+Concern (delay).
+Piling work for the Cooling Tower may affect Metek Company due to vibrations impacting its X-ray measuring equipment.
+CEEC has held discussions with Metek Company to obtain approval for the piling work to proceed.
+Safety &amp; Health
+Management Weekly Route Walk - Every Tuesday
+Weekly ESH Meeting - Every Tuesday
+Weekly Project Meeting with - Every Tuesday</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>PRJ-016</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>MKP</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="2" t="inlineStr"/>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Bunker Pit Wall to +5.45 EL
+Bunker Building ground level construction
+Boiler structure construction
+Flue gas treatment structure construction
+STG&amp;EC Building construction
+Underground Piping work
+Pile Driving for Tipping Area
+Duct bank and Cathodic protection installation
+Concern (delay)
+Manpower shortage
+Late manufacturing for steel roof structure and cladding structure
+Accuracy of embedded plate installation
+Secondary Beam – Location Change
+Underground pipes are required long lead for fabrication and delivery from oversea manufacturer. (Steel pipe 24”&amp;28”)
+1 Duct bank and Cathodic protection drawing were not finalized
+2 Delay of Material purchasing.
+SEPEC/STECON is requested to increase the workforce to maintain the schedule.
+Follow-up CEEC/SEPEC to urgently conclude the detail of steel roof structure and cladding structure
+SEPEC/STECON are required to ensure embedded plates are installed at the correct elevation
+SEPEC to confirm the changing of the secondary beam location.</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>(19 Jun 26) (26 Jun 26)
+Activities CC/SC (*)
+Plan Actual Diff. Plan Actual Diff. Acc.Plan
+% % % % % % %
+Engineering 10% 49.18 42.00 -7.18 53.60 44.40 -9.20 60.16
+Procurement 40% 65.88 63.65 -2.23 67.82 65.44 -2.38 69.36
+Construction 40% 7.14 8.29 1.15 8.21 8.89 0.68 9.01
+Commissioning 10% 0 0 0 0 0 0 0
+Overall 100% 34.13 32.98 -1.15 35.77 34.17 -1.60 37.36
+Safety &amp; Health :
+• Conduct SafetyToolbox Talk before starting work.
+• Mass Safety Talk at Site Area
+• Management Walk Down every Friday (10.00 – 11.00)
+• HSE Weekly Audit every Wednesday (10.00-11.00)
+• HSE Weekly Meeting with Subcontractor every Wednesday (10.00-11.00)
+• Safety Induction Training for newcomers
+• Working at height Training
+Environment &amp; CoP :
+• Water spray at construction site
+• Temporary Wheel wash station</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>PRJ-017</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>MPE</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr"/>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>248 Incinerator Arrival at site 21 May 26 28 May 26 Planned delivery to site on 11/07
+253 Steam turbine Arrivalat site 22 Dec 26 29 Dec 26
+609 Producing qualified water (Water Receiving date) 8 May 27 21 May 27
+EPC has adjusted the PMS to Rev.C to make the plan consistent with the actual work.
+➢ Boiler foundation construction
+➢ Steam Turbine Generator &amp; Electrical Construction
+Concern (delay)
+Tasks that have started and those that have not yet started are behind schedule (PMS plan).
+Follow-up work with catch-up plan by daily.
+Inform EPC to Boiler focus H/O 8/12 pole on 17 Jul 26
+Expedite to EPC&amp; STECON increase manpower.
+Follow –up manpower with STECON in weekly and daily meeting.
+Expediting STECON to do work with catch-up plan by daily
+Plan to do parallel work .
+Safety Weekly Audit issue status by weekly
+Total Issues
+since 02 Apr 2026 - Present 10
+(Every Tuesday morning) 4
+4-Jun-26 11-Jun-26 18-Jun-26 25-Jun-26
+Safety Audit issue Status Chart Open Closed</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Safety &amp; Health:
+Management site walkdown
+Toolbox talk activity
+Safety induction training to new contractors​
+Weekly Inspect Safety​
+Weekly Random Alc. Test
+Environment &amp; CoP:
+Road cleaning (Campsite STECON/IEAT Road)
+Water spray to reduce dust
+Monitor noise during overtime work
+Activities CC/SC (*)
+Plan Actual Diff. Plan Actual Diff. Acc.Plan
+% % % % % % %
+Engineering 10.00% 45.80% 42.11% -3.69% 49.27% 44.09% -5.18% 53.05%
+Procurement 40.00% 47.48% 54.24% 6.76% 50.28% 58.17% 7.89% 52.58%
+Construction 40.00% 4.85% 6.05% 1.20% 5.22% 6.33% 1.11% 5.64%
+Commissioning 10.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00%
+Overall 100.00% 25.51% 28.32% 2.81% 27.13% 30.21% 3.08% 28.59%
+** The data cut off every Friday of week.
+On Schedule A Bit Delay Big Delay</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>PRJ-018</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>PFP</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="2" t="inlineStr"/>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Boiler foundation construction work.
+Steam Turbine Generator &amp; Electrical Construction work .
+Concern (Delay)
+Tasks that have started and those that have not yet started are behind schedule (PMS plan)
+• Follow-up work with catch-up plan by daily
+• Inform EPC to Boiler focus H/O 8/12 pole on 7 Jul 26
+• Follow –up manpower with STECON in daily meeting
+• Expediting STECON to do work with catch-up plan by daily
+• Plan to do parallel work and reduce duration time some step of work.
+Safety Weekly Audit issue status by weekly
+Total Issues
+since 02 Apr 2026 - Present 20
+(Every Tuesday morning)
+4-Jun-26 11-Jun-26 18-Jun-26 25-Jun-26
+Open Closed
+Safety Audit issue Status Chart
+and anxieties.
+Environmental Impact Assessment -Environment Impact Assessment At least twice SM ,CR and -
+Done 27 May 2026
+Committee meeting. Committee a year SSHE</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Safety &amp; Health:
+Management site walkdown
+Toolbox talk activity
+Safety induction training to new contractors​
+Weekly Inspect Safety​
+Weekly Random Alc. Test
+Environment &amp; CoP:
+Road cleaning (Campsite STECON/IEAT Road)
+Water spray to reduce dust
+Monitor noise during overtime work
+Activities CC/SC (*)
+Plan Actual Diff. Plan Actual Diff. Acc.Plan
+% % % % % % %
+Engineering 10.00% 49.18% 42.26% -6.92% 53.60% 44.50% -9.10% 60.16%
+Procurement 40.00% 65.88% 63.65% -2.23% 67.82% 65.44% -2.38% 69.36%
+Construction 40.00% 7.14% 6.61% -0.53% 8.21% 6.98% -1.23% 9.01%
+Commissioning 10.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00%
+Overall 100.00% 34.13% 32.33% -1.80% 35.77% 33.42% -2.35% 37.36%
+** The data cut off every Friday of week.
+** Procurement delay from Manufacturing Boiler structure &amp; equipment and Manufacturing STG foundation anchor bolts, condenser metal sheet</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>PRJ-019</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>PKP</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr"/>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Completion of Bunker Building Concrete pouring Lift 1 Wall -5.7 to +1.0 EL ; (First step is to pour concrete up to kicker level on 1-2 Jul ; the second step is
+to pour the concrete up to +1.00 EL on 30-31 Jul
+CEEC/STECON will hand over the main 8 column pedestals (excluding the ground base slab) of the Boiler on 13-JUL- 2026 for HUASHI to perform
+the first lift of the steel structure on 14-JUL-2026. The remaining 4 column pedestals in the boiler area must be handed over to Huashi within 7 days
+on 20-JUL-2026 of the handover of the above columns.
+Concern(delay)
+Limited site access roads may impact construction productivity and material logistics.
+The Owner coordinated with CEEC and STECON to find a solution.
+61 Safety Weekly Audit issue status by weekly
+Total Issues 10
+Since 25 Jan 2026
+Safety Weekly Audit issue Status Chart
+Open Closed
+Before After
+The electrical outlet cover is Already improved.
+Government Agencies
+Area of concern :
+Access road obstruction with construction STG Building.
+• The Owner coordinated with CEEC and STECON to find a troubleshooting solution.
+• Access road obstruction with construction STG Building.</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Catch-up plan for the partial handover of the FGT area, to HUASI erection work is under review by
+TRIR 0 CEEC and is expected to be submitted on 3 July 2026.
+Key Lookahead Milestones:
+Bunker Building: Lift 1 (-5.7 to +1.0 EL). The first step is to pour concrete up to kicker level on 1–2
+Jul. The second step is to pour concrete up to +1.0 m on 30–31 Jul (Completed Lift-1)
+Boiler Island Area: Partial handover (Z1-Z4), followed by pedestal and tie beam concrete pouring.
+Area of Concern:
+Bunker, Boiler, FGT &amp; STG Installation: Level 3 schedule update from CEEC is still pending.
+Limited site access roads may impact construction productivity and material logistics.
+Issue to request HO support:
+Safety &amp; Health
+Management Weekly Route Walk - Every Tuesday
+Weekly ESH Meeting - Every Tuesday
+Weekly Project Meeting with - Every Tuesday
+Toolbox Talk - Everyday before working
+Safety training (if any)
+Inspect equipment before working (Daily)
+Random test alcohol
+Environment &amp; CoP
+Road cleaning.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>PRJ-020</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>PSD</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="2" t="inlineStr"/>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Completion of Bunker Building Concrete pouring Lift 1 Wall -5.7 to +1.0 EL ; (First step is to pour concrete up to kicker level on 1-2 Jul ; the second
+step is to pour the concrete up to +1.00 EL on 15-16 Jul
+CEEC/STECON will hand over the main 8 column pedestals (excluding the ground base slab) of the Boiler on 6th of July 2026 for HUASHI to perform
+the first lift of the steel structure on 7-JUL-2026. The remaining 4 column pedestals in the boiler area must be handed over to Huashi within 7 days
+on 14-JUL-2026 of the handover of the above columns.
+Partial handover (civil works) of Switchgear room in the STG &amp; EC Building, including all related areas required for the installation of 22 kV and 11 kV
+switchgear and power cables.
+Note : Bunker, Boiler, FGT &amp; STG Installation: The Level 3 schedule update from CEEC is still pending. CEEC has committed to submitting the schedule
+70 Safety Weekly Audit issue status by weekly
+Total Issues
+Since 2 Jan 2026 5
+18 - 24 June
+Safety Weekly Audit issue Status Chart
+Open Closed
+Before After
+Concrete poor waste Already improved
+Government Agencies
+Problem : Electric Pole obstruct Entrance
+ต ำแหน่งเสำไฟฟ้ำเดมิ
+N.= 1602494.440</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Concern (delay) : None
+Safety &amp; Health
+Management Weekly Route Walk - Every Tuesday
+Weekly ESH Meeting - Every Tuesday
+Weekly Project Meeting with - Every Tuesday
+Toolbox Talk - Everyday before working
+Safety training (if any)
+Inspect equipment before working (Daily)
+Random test alcohol
+Environment &amp; CoP
+Road cleaning.
+Water spray to reduce dust 2 times/day
+Visual inspect storm drainage
+Housekeeping
+• ERC Audit on 29th June 2026
+Jun 2026) Jun 2026)
+Activities CC/SC (*)
+Plan Actual Diff. Plan Actual Diff. Acc.Plan
+% % % % % % %
+Engineering 10% 67.58% 42.87% -24.71% 74.32% 44.38% -29.94% 90.50%</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>PRJ-021</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>PWW1</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="2" t="inlineStr"/>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Back Energize Work
+Retaining wall (PWW1, 2) - Final drawing
+Water treatment plant (Clarifier)
+Service water storage (สว นทเ่ี ปน Tank เหลก็ )
+Fire pump room (แบบยังไมครบ ตองการแบบพ(cid:245)้น เสา คาน งานเหล็กรูปพรรณและแบบสถาปตย)
+Transformer (Foundation + Fire wall) - ยงั ไมม แี บบ
+Bunker wall opening/conveyor belt
+(cid:341) (cid:341) (cid:341)
+มเี รอื ง cable duct ไม่ม ี duct bank structural detail STECON แจง้ ว่าไม่สามารถใชส้ งั ของและสงั จา้ ง ผรม ได้
+Refuse Bunker foundation construction work
+Boiler Island foundation construction
+STG Building construction
+Follow up EPC to revise the catch-up plan and monitor work progress.
+Increase overtime activities and inform neighbors about the plan.
+Expedite for Method Statement/ Engineering drawing
+Revise the catch-up plan and monitor work progress.
+90 Safety Weekly Audit issue status by weekly
+Total Issues 40
+Since 2 Apr 2026
+Safety Weekly Audit issue Status Chart</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Safety &amp; Health:
+(cid:127) Safety Toolbox Talk before starting work and Mass Safety Talk.
+(cid:127) Safety induction training.
+(cid:127) Tools and equipment’s inspection.
+(cid:127) Management walkdown.
+(cid:127) Random alcohol test.
+(cid:127) Random drug test.
+Environment &amp; CoP:
+(cid:127) Water spray to reduce dust.
+(cid:127) Wheel washing before entering public road.
+(cid:127) Road cleaning.
+(cid:127) Prepare for LTA&amp;ADB audit.
+WAdadll +w5a.l4l 5fo mr .c toon +v1e8y.o3r5 b mel.t (Use slipform) (cid:127) Bunker wall
+(WaiStitnagrt c Jounlyfi trom e DndW oGf .1)5 Sep 26 (cid:127) Continuous backfill work
+(cid:127) Continuous install rebar work
+(cid:127) Start slipform surveying at the steel former warehouse.
+(cid:127) Rebar work –Lack of manpower
+(cid:127) Steconallocate worker to boiler and STG building area so no manpower
+Wall 2ndstep to +5.45 m. (Use jump form) for start rebar work. (Resume rebar work on 22 June 26)
+Plan 20 July 26 (cid:127) The opening maybe change concept (Reduce from 3 to 2 because will use for</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>PRJ-022</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>PWW2</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="2" t="inlineStr"/>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Refuse Bunker foundation construction work
+Boiler Island foundation construction
+STG foundation construction
+Follow up catch up plan
+Expedite for Method Statement/ Engineering drawing
+48 Safety Weekly Audit issue status by weekly
+Total Issues
+Since 2 Apr 2026
+0 0 0 0 0 02
+April'26 May'26 4-10 Jun '26 11-17 Jun'26 18-24 Jun'26
+Safety Weekly Audit issue Status Chart
+Open Closed
+Safety sign
+BEFORE AFTER
+PWW Access road
+o Follow up Access Road Drawing and comment Drawing.
+(cid:127) Follow up CEEC &amp; STECON Order Material of piping.&gt;&gt;Still STECON Request a price from the seller.
+(cid:127) Follow up CEEC Eng. Change sizing of STW Pipe from 16’ to 12’ and ask CEEC Expedite submit new version
+of PWW Access Road General Layout Drawing.&gt;&gt; Already change to 12”.
+Fire water system</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Safety &amp; Health:
+(cid:127) Safety Toolbox Talk before starting work and Mass Safety Talk.
+(cid:127) Safety induction training.
+(cid:127) Tools and equipment’s inspection.
+(cid:127) Management walkdown.
+(cid:127) Random alcohol test.
+(cid:127) Random drug test.
+Environment &amp; CoP:
+(cid:127) Water spray to reduce dust.
+(cid:127) Wheel washing before entering public road.
+(cid:127) Road cleaning.
+(cid:127) Prepare for LTA&amp;ADB audit.
+(cid:127) Refuse bunker wall
+(cid:127) Continuous remove formwork
+Concrete wall +1.00 m. (cid:127) Install waterproof membrane
+(Complete) (cid:127) Bunker building
+(cid:127) Continuous Install rebar, formwork and pouring concrete surrounding column
+Activity Qty total Qty complete %Complete
+Bunker wall –Formwork 1000 sq.m. 1000 sq.m. 100.00%
+Bunker wall –Concrete 300 cu.m. 300 cu.m 100.00%</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>PRJ-023</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>TPP</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="2" t="inlineStr"/>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Bunker Pit Wall to +8.00 EL
+Bunker Building ground level construction
+Boiler structure construction
+Flue Gas Treatment structure construction
+STG&amp;EC Building construction
+Underground Piping work
+Incinerator steel structure installation
+Ground floor level construction for Tipping Area
+Duct bank and Cathodic protection installation
+Concern (delay)
+Feeding gate installation may be delayed, as the building at EL +7.95 is planned to finish slab concrete on 31/7/26.
+STECON will pour the concrete slab partially due to the missing underground drawing.
+FGT Foundation – Holding Cloud
+The 'up to ground level' completion milestone has been revised from 15/6/26 to 7/7/26.
+Underground pipes are required long lead for fabrication and delivery from oversea manufacturer. (Steel pipe 24”&amp;28”)
+1 Duct bank and Cathodic protection drawing were not finalized
+2 Delay of Material purchasing.
+STECON clarified that the work will catch up with the working plan at the floor EL +4.25m activity.
+SEPEC to confirm the underground drawing.
+SEPEC is to confirm the holding cloud mark in the FGT foundation drawing.</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>(19 Jun 26) (26 Jun 26)
+Activities CC/SC (*)
+Plan Actual Diff. Plan Actual Diff. Acc.Plan
+% % % % % % %
+Engineering 10% 67.58 42.52 -25.06 74.32 44.08 -30.24 80.30
+Procurement 40% 71.12 69.35 -1.77 72.89 70.86 -2.03 74.39
+Construction 40% 13.16 11.76 -1.40 14.29 12.26 -2.03 15.70
+Commissioning 10% 0 0 0 0 0 0 0
+Overall 100% 40.47 36.70 -3.77 42.30 37.66 -4.64 44.06
+Safety &amp; Health :
+• Conduct SafetyToolbox Talk before starting work.
+• Mass Safety Talk at Site Area
+• Management Walk Down every Friday (10.00 – 11.00)
+• HSE Weekly Audit every Wednesday (10.00-11.00)
+• HSE Weekly Meeting with Subcontractor every Wednesday (10.00-11.00)
+• Safety Induction Training for new comers
+• Working at height Training
+Environment &amp; CoP :
+• Water spray at construction site
+• Temporary Wheel wash station</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>PRJ-024</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>TSE</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr"/>
-      <c r="E23" s="2" t="inlineStr"/>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Bunker and surrounding: Foundation up to ground (including the surrounding room, underground grounding system).
+Boiler : Boiler steel structure.
+Flue gas treatment : Foundation work. Start steel structure erection
+STG &amp; ECB : Foundation up to ground (including the surrounding room, underground grounding system).
+Tipping hall: Pilling work and foundation.
+Concern (delay)
+Delay finish of bunker foundations up to ground level. Target on PMS 08 May 2026.
+Delay finish of STG foundations up to ground level. Target on PMS 08 Jun 2026.
+CEEC/STECON prepared catch-up plan for bunker and follow up
+CEEC/STECON will increase man power more than plan
+- This week (Finished : 8)
+- Total(Finished : 50)
+0 RFC , 3 NCR
+7 Stakeholder Engagement Plan Continue as plan
+8 SHE Plan for counting manpower working at site Manpower daily report have started to generating automatically at 7:00
+AM everyday by e-mail
+9 Status of EPC Foreigner staff and worker personal mandatory document Pending 27 prs. Plan to finish &lt;10 Jul 2026&gt;
+50 Safety Weekly Audit issue
+Total Issues
+(Since 2 Apr 2026 onwards)</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Activities CC/SC (*)
+Plan% Actual% Diff.% Plan% Actual% Diff.% Acc.Plan%
+Engineering 10% 81.62% 48.01% -33.61% 86.57% 49.55% -37.02% 88.00%
+Procurement 40% 77.41% 74.49% -2.92% 79.32% 75.53% -3.79% 80.86%
+Construction 40% 14.79% 14.66% -0.13% 16.34% 15.23% -1.11% 18.06%
+Commissioning 10% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00%
+Overall 100% 45.04% 40.46% -4.58% 46.92% 41.26% -5.66% 48.37%
+5 Maximum Quantity of Heavy Machinery at Site Inspection as period
+and keep related document
+6 Summary of SHE Weekly Audit issues Walk down
+- This week (Finished : 8)
+- Total(Finished : 50)
+0 RFC , 3 NCR
+7 Stakeholder Engagement Plan Continue as plan
+8 SHE Plan for counting manpower working at site Manpower daily report have started to generating automatically at 7:00
+AM everyday by e-mail
+9 Status of EPC Foreigner staff and worker personal mandatory document Pending 27 prs. Plan to finish &lt;10 Jul 2026&gt;
+Safety &amp; Health:
+• Safety Toolbox Talk before starting work and Mass Toolbox Talk and counting manpower
+• Safety training for newcomer</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">

</xml_diff>